<commit_message>
Updated Graphics - Specular
</commit_message>
<xml_diff>
--- a/Assets/Level ideas.xlsx
+++ b/Assets/Level ideas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osama-App\Documents\Unity Projects\Matryoshka Puzzle\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8B47B7-C6ED-49CD-AE48-63113436C3A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576A1F94-86FA-4455-8910-7F16AB937FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D7CD07F5-B6A9-4E1A-9152-6758E6D251FF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Level</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>Testing general understanding</t>
-  </si>
-  <si>
-    <t>Blocked tiles</t>
   </si>
   <si>
     <t>Buttons to unlock blocked tiles</t>
@@ -489,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43240939-9CA8-490C-880F-4AC6927310CD}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
@@ -557,7 +554,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -613,7 +610,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -621,7 +618,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -685,7 +682,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -693,15 +690,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>